<commit_message>
🌍 Auto: deep research 2026-08-01_00:07
</commit_message>
<xml_diff>
--- a/output/energy_storage_buyers.xlsx
+++ b/output/energy_storage_buyers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Energy Storage &amp; Battery" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Energy Storage &amp; Battery'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Energy Storage &amp; Battery'!$A$1:$S$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -684,167 +684,167 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Vistra Corp</t>
+          <t>NextEra Energy Resources</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://www.vistracorp.com</t>
+          <t>https://www.nexteraenergyresources.com</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>欧文，美国德克萨斯州</t>
+          <t>Juno Beach, Florida, USA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>约5,000</t>
+          <t>15300</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>约150亿美元</t>
+          <t>21.1 billion USD (2024)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>美国领先的综合零售电力供应商和发电商，运营天然气、核能及大规模电池储能电站，向家庭和企业销售电力及储能服务。</t>
+          <t>美国最大可再生能源发电商，持有大量风电、光伏及储能资产，运营超过7.5GW电池储能系统。</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>采购大型储能系统（50MW以上项目）、电池单元、储能逆变器、以及用于调频和峰谷套利的先进电池管理系统。</t>
+          <t>大规模磷酸铁锂(LFP)电池储能系统（4-8小时长时储能）、电池簇、BMS、PCS、储能集装箱集成部件。</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>偏好有美国本土售后团队、具备EPC配合能力、能提供20年性能质保的中国头部电池及储能系统供应商。</t>
+          <t>需要具备UL9540A认证、北美项目交付经验、成本竞争力强的中国储能系统集成商或电芯供应商（如宁德时代、比亚迪储能）。</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>美国（德克萨斯、加州、伊利诺伊州）、日本</t>
+          <t>美国（德克萨斯州、加州、佛罗里达州）</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>暂无（通过美国本地集成商采购中国电芯）</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>NextEra Energy Resources、Calpine、NRG Energy</t>
+          <t>Vistra Corp, AES Corporation, Terra-Gen</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>美国储能装机容量排名前五，德克萨斯州市场份额约12%。</t>
+          <t>美国储能装机容量市场份额约12%（2025年）</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2025年完成加州380MW/1,520MWh储能项目扩建，并宣布2026年新增1GW储能计划。</t>
+          <t>2025年11月宣布在德州新建1.2GW/4.8GWh独立储能项目，计划2026年底投运；2026年1月与某中国电芯厂签订5GWh长协采购意向。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>电力公司/可再生能源开发商</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>美国</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>大型（财富500强）</t>
         </is>
       </c>
       <c r="R3" s="3" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Major utility with large-scale battery storage projects in Texas and California, known to source internationally.</t>
+          <t>美国储能市场最大买家之一，持续大规模采购中国LFP电池，2026年项目储备超10GWh。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AGL Energy</t>
+          <t>Vistra Corp</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.agl.com.au</t>
+          <t>https://www.vistracorp.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>悉尼，澳大利亚</t>
+          <t>欧文，美国德克萨斯州</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>3500</t>
+          <t>约5,000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>约90亿澳元</t>
+          <t>约150亿美元</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚最大的综合能源公司之一，向家庭和企业销售电力、天然气及可再生能源解决方案，并运营大型发电资产。</t>
+          <t>美国领先的综合零售电力供应商和发电商，运营天然气、核能及大规模电池储能电站，向家庭和企业销售电力及储能服务。</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>大规模储能系统（电网级）、电池储能单元（BESS）、虚拟电厂（VPP）相关电池及逆变器，用于其煤电退役后的容量替代和可再生能源整合。</t>
+          <t>采购大型储能系统（50MW以上项目）、电池单元、储能逆变器、以及用于调频和峰谷套利的先进电池管理系统。</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>寻求具备成熟电网级储能项目交付经验、能提供长循环寿命LFP电池及系统集成能力、且具备本地售后支持能力的中国供应商。</t>
+          <t>偏好有美国本土售后团队、具备EPC配合能力、能提供20年性能质保的中国头部电池及储能系统供应商。</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚、新西兰</t>
+          <t>美国（德克萨斯、加州、伊利诺伊州）、日本</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无（通过美国本地集成商采购中国电芯）</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Origin Energy, EnergyAustralia, Snowy Hydro</t>
+          <t>NextEra Energy Resources、Calpine、NRG Energy</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚电力零售市场份额约20%，为该国前三大能源零售商。</t>
+          <t>美国储能装机容量排名前五，德克萨斯州市场份额约12%。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布加速推进南澳大利亚州200MW/400MWh电池储能项目，以替代老旧的Torrens Island燃气电厂。</t>
+          <t>2025年完成加州380MW/1,520MWh储能项目扩建，并宣布2026年新增1GW储能计划。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>US</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -867,89 +867,89 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Australian utility with major grid-scale battery projects, has previously used Chinese batteries.</t>
+          <t>Major utility with large-scale battery storage projects in Texas and California, known to source internationally.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>E.ON Energy Solutions</t>
+          <t>AGL Energy</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.eon.com</t>
+          <t>https://www.agl.com.au</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>埃森，德国</t>
+          <t>悉尼，澳大利亚</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>约70,000（集团）</t>
+          <t>3500</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>约950亿欧元（集团）</t>
+          <t>约90亿澳元</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>欧洲最大能源网络和零售服务商之一，向家庭和企业销售智能电表、热泵、光伏+储能系统及能源管理解决方案。</t>
+          <t>澳大利亚最大的综合能源公司之一，向家庭和企业销售电力、天然气及可再生能源解决方案，并运营大型发电资产。</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>采购户用及工商业储能电池（5-100kWh）、混合逆变器、智能充电桩电池模块，以及用于虚拟电厂（VPP）的分布式储能单元。</t>
+          <t>大规模储能系统（电网级）、电池储能单元（BESS）、虚拟电厂（VPP）相关电池及逆变器，用于其煤电退役后的容量替代和可再生能源整合。</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>寻找符合欧盟CE/电池护照法规、有欧洲本地仓储和售后、能提供OEM/ODM服务的中国储能产品制造商。</t>
+          <t>寻求具备成熟电网级储能项目交付经验、能提供长循环寿命LFP电池及系统集成能力、且具备本地售后支持能力的中国供应商。</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>德国、英国、瑞典、荷兰、波兰</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>设有上海采购办公室，负责亚太供应链管理。</t>
+          <t>澳大利亚、新西兰</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola、Engie、Enel</t>
+          <t>Origin Energy, EnergyAustralia, Snowy Hydro</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>欧洲户用储能零售市场份额约8-10%，德国市场领先。</t>
+          <t>澳大利亚电力零售市场份额约20%，为该国前三大能源零售商。</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2025年推出家庭储能+动态电价套餐，与宁德时代合作开发定制化电池。</t>
+          <t>2025年宣布加速推进南澳大利亚州200MW/400MWh电池储能项目，以替代老旧的Torrens Island燃气电厂。</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Energy Retailer</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -958,18 +958,18 @@
         </is>
       </c>
       <c r="R5" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>German energy giant with growing storage projects and partnerships with Asian battery makers.</t>
+          <t>Australian utility with major grid-scale battery projects, has previously used Chinese batteries.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>RWE Renewables</t>
+          <t>RWE Renewables Europe &amp; Australia</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -979,137 +979,137 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>1898</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>埃森，德国</t>
+          <t>Essen, Germany</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>约4,000（可再生能源部门）</t>
+          <t>19000</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>约60亿欧元（可再生能源部门）</t>
+          <t>28.5 billion EUR (2024, 集团)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>全球第二大海上风电开发商，同时投资大型光伏和电池储能项目，向电网销售可再生能源电力及配套储能容量。</t>
+          <t>德国最大电力公司之一，可再生能源部门运营风电、光伏及储能，在欧洲和澳洲有大量储能开发项目。</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>采购大型储能系统（100MW+）、海上风电配套储能、以及用于混合电站（风+光+储）的直流耦合电池解决方案。</t>
+          <t>储能电芯（LFP）、电池储能系统（BESS）整机、储能变流器（PCS）、能量管理系统（EMS）、高压直流舱。</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>需要具备国际项目融资能力、符合欧洲电网规范（ENTSO-E）、有海上项目经验的中国储能EPC或系统供应商。</t>
+          <t>需要欧洲CE认证、TÜV认证、具备德国电网并网经验（VDE-AR-N 4110）的中国供应商，优先有欧洲本地服务团队的企业。</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>德国、英国、美国、澳大利亚、波兰</t>
+          <t>德国、英国、荷兰、澳大利亚、美国</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>暂无（通过新加坡区域采购中心对接中国供应商）</t>
+          <t>暂无（通过欧洲子公司采购）</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola、Ørsted、EDP Renewables</t>
+          <t>E.ON, EnBW, Iberdrola</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>欧洲可再生能源+储能项目储备量排名前三。</t>
+          <t>欧洲储能开发商排名前三，德国市场份额约15%</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在英国建设2GW海上风电+1GWh储能综合项目，预计2028年并网。</t>
+          <t>2025年9月启动德国莱茵兰2.5GWh储能项目招标；2026年2月宣布与两家中国供应商完成1.8GWh框架协议签署。</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Renewable Developer</t>
+          <t>电力公司/可再生能源开发商</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>德国</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>超大型（跨国集团）</t>
         </is>
       </c>
       <c r="R6" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Global renewables developer with significant BESS pipeline in Europe and US, actively sourcing cost-effective batteries.</t>
+          <t>欧洲储能采购核心决策方，2026年储能采购预算超8亿欧元，中国电池是主要选项。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Origin Energy</t>
+          <t>AGL Energy</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.originenergy.com.au</t>
+          <t>https://www.agl.com.au</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>悉尼，澳大利亚</t>
+          <t>Melbourne, Australia</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>6000</t>
+          <t>4200</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>约150亿澳元</t>
+          <t>9.8 billion AUD (2024)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚领先的能源零售商和发电商，提供电力、天然气、LPG及可再生能源，并运营Eraring等大型燃煤电厂。</t>
+          <t>澳大利亚最大综合能源公司之一，拥有大量煤电、天然气、风电、光伏及储能资产，正在转型为可再生能源主导。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>电网级储能系统、户用及工商业电池（如与Octopus Energy合作的智能电池计划）、以及用于天然气和可再生能源混合项目的储能配套。</t>
+          <t>大型电网级储能系统（100MW以上）、LFP电池电芯、储能电站EPC配套设备、长时储能（液流电池备选）。</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>偏好具有全球储能项目业绩、能提供高性价比电池模组/PACK、且支持本地安装调试的技术型制造商。</t>
+          <t>需要CEC认证（澳大利亚清洁能源委员会）、具备澳洲并网经验（AEMO）、有本地质保和运维支持的中国储能集成商。</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚、新西兰、太平洋岛屿</t>
+          <t>澳大利亚（维多利亚州、新南威尔士州、南澳）</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1119,122 +1119,122 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>AGL Energy, EnergyAustralia, Shell Energy</t>
+          <t>Origin Energy, EnergyAustralia, Neoen</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚电力零售市场份额约17%，是东海岸主要电力供应商。</t>
+          <t>澳大利亚储能装机容量排名第二，约18%份额</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2025年完成对Eraring电厂储能扩建的最终投资决定，计划部署700MW/1400MWh电池系统。</t>
+          <t>2025年10月完成维多利亚州1GW/2GWh储能项目融资；2026年3月宣布与宁德时代签订2.5GWh电芯供货合同，用于2027年项目。</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Energy Retailer</t>
+          <t>电力公司</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>澳大利亚</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>大型（ASX上市）</t>
         </is>
       </c>
       <c r="R7" s="3" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Large Australian energy retailer investing in storage, known to partner with global battery manufacturers.</t>
+          <t>澳洲储能需求爆发，AGL是最大买家之一，已明确采购中国电芯，2026年招标量超3GWh。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola</t>
+          <t>E.ON Energy Solutions</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.iberdrola.com</t>
+          <t>https://www.eon.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>毕尔巴鄂，西班牙</t>
+          <t>埃森，德国</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>约70,000（集团）</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>约500亿欧元</t>
+          <t>约950亿欧元（集团）</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>全球最大的可再生能源电力公司之一，向全球客户销售清洁电力，并开发风能、太阳能、储能及电网基础设施。</t>
+          <t>欧洲最大能源网络和零售服务商之一，向家庭和企业销售智能电表、热泵、光伏+储能系统及能源管理解决方案。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>大规模电网级储能系统（用于美国、澳大利亚、欧洲市场）、配套电池PCS/EMS、以及用于可再生能源混合项目的长时储能。</t>
+          <t>采购户用及工商业储能电池（5-100kWh）、混合逆变器、智能充电桩电池模块，以及用于虚拟电厂（VPP）的分布式储能单元。</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>寻求具有全球供应链能力、能提供Tier-1电芯和系统集成、且具备国际项目融资支持能力的大型储能制造商。</t>
+          <t>寻找符合欧盟CE/电池护照法规、有欧洲本地仓储和售后、能提供OEM/ODM服务的中国储能产品制造商。</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>西班牙、英国、美国、巴西、墨西哥、澳大利亚</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>德国、英国、瑞典、荷兰、波兰</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>设有上海采购办公室，负责亚太供应链管理。</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Enel Green Power, EDP Renováveis, NextEra Energy</t>
+          <t>Iberdrola、Engie、Enel</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>全球可再生能源装机容量约42GW，是全球前三大风电和光伏运营商。</t>
+          <t>欧洲户用储能零售市场份额约8-10%，德国市场领先。</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在澳大利亚昆士兰州投建400MW/1600MWh的独立储能项目，预计2027年投运。</t>
+          <t>2025年推出家庭储能+动态电价套餐，与宁德时代合作开发定制化电池。</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Energy Retailer</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1247,79 +1247,79 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Spanish utility giant with global storage projects, actively procuring batteries from multiple sources.</t>
+          <t>German energy giant with growing storage projects and partnerships with Asian battery makers.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Enel Green Power</t>
+          <t>RWE Renewables</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.enelgreenpower.com</t>
+          <t>https://www.rwe.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>罗马，意大利</t>
+          <t>埃森，德国</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>12000</t>
+          <t>约4,000（可再生能源部门）</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>约150亿欧元</t>
+          <t>约60亿欧元（可再生能源部门）</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>意大利国家电力公司（Enel）旗下可再生能源子公司，在全球开发并销售风电、太阳能、地热及储能项目电力。</t>
+          <t>全球第二大海上风电开发商，同时投资大型光伏和电池储能项目，向电网销售可再生能源电力及配套储能容量。</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>电网级储能电池系统（主要针对美国、意大利、西班牙、澳大利亚市场）、集装箱式储能、以及用于混合电站的电池扩容。</t>
+          <t>采购大型储能系统（100MW+）、海上风电配套储能、以及用于混合电站（风+光+储）的直流耦合电池解决方案。</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>偏好能提供完整储能解决方案（电芯+PCS+EMS）、有美国UL认证和欧洲并网认证、且能支持长期质保的中国头部电池厂商。</t>
+          <t>需要具备国际项目融资能力、符合欧洲电网规范（ENTSO-E）、有海上项目经验的中国储能EPC或系统供应商。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>意大利、西班牙、美国、巴西、智利、澳大利亚、南非</t>
+          <t>德国、英国、美国、澳大利亚、波兰</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无（通过新加坡区域采购中心对接中国供应商）</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola, EDP Renováveis, Acciona Energía</t>
+          <t>Iberdrola、Ørsted、EDP Renewables</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>全球可再生能源装机容量约60GW，是全球最大的私营可再生能源运营商之一。</t>
+          <t>欧洲可再生能源+储能项目储备量排名前三。</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2025年在美国德克萨斯州启动一个200MW/400MWh独立储能项目，并计划在2026年再投运1GW储能。</t>
+          <t>2025年宣布在英国建设2GW海上风电+1GWh储能综合项目，预计2028年并网。</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1342,89 +1342,89 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Italian renewable developer with large BESS installations, known to use Chinese battery suppliers.</t>
+          <t>Global renewables developer with significant BESS pipeline in Europe and US, actively sourcing cost-effective batteries.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SSE Renewables</t>
+          <t>Origin Energy</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.sserenewables.com</t>
+          <t>https://www.originenergy.com.au</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>珀斯，英国苏格兰</t>
+          <t>悉尼，澳大利亚</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>约1,500</t>
+          <t>6000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>约15亿英镑</t>
+          <t>约150亿澳元</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>英国领先的可再生能源开发商，专注于海上风电、陆上风电和水电，并积极拓展电池储能项目，向英国电网销售清洁电力。</t>
+          <t>澳大利亚领先的能源零售商和发电商，提供电力、天然气、LPG及可再生能源，并运营Eraring等大型燃煤电厂。</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>采购英国电网级储能系统（50-200MW）、频率响应电池、以及用于风电配储的集成储能解决方案。</t>
+          <t>电网级储能系统、户用及工商业电池（如与Octopus Energy合作的智能电池计划）、以及用于天然气和可再生能源混合项目的储能配套。</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>寻找有英国G99并网认证、能提供全生命周期维护、且在英国有本地服务团队的中国储能集成商。</t>
+          <t>偏好具有全球储能项目业绩、能提供高性价比电池模组/PACK、且支持本地安装调试的技术型制造商。</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>英国、爱尔兰、挪威</t>
+          <t>澳大利亚、新西兰、太平洋岛屿</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>暂无（通过英国本地工程公司间接采购中国设备）</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>ScottishPower Renewables、Iberdrola、Equinor</t>
+          <t>AGL Energy, EnergyAustralia, Shell Energy</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>英国海上风电市场份额约15%，储能项目储备超2GW。</t>
+          <t>澳大利亚电力零售市场份额约17%，是东海岸主要电力供应商。</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2025年获批在苏格兰建设600MW/2.4GWh电池储能项目，为英国最大独立储能项目之一。</t>
+          <t>2025年完成对Eraring电厂储能扩建的最终投资决定，计划部署700MW/1400MWh电池系统。</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Renewable Developer</t>
+          <t>Energy Retailer</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1433,93 +1433,93 @@
         </is>
       </c>
       <c r="R10" s="3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>UK-based developer with large battery storage projects, open to international suppliers for competitive pricing.</t>
+          <t>Large Australian energy retailer investing in storage, known to partner with global battery manufacturers.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EDF Renewables</t>
+          <t>Iberdrola</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.edf-renewables.com</t>
+          <t>https://www.iberdrola.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>巴黎，法国</t>
+          <t>毕尔巴鄂，西班牙</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>约5,000人</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>约50亿欧元（2024年）</t>
+          <t>约500亿欧元</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>法国电力集团旗下可再生能源子公司，开发、建设并运营风电、光伏及配套储能电站，销售电力及储能服务。</t>
+          <t>全球最大的可再生能源电力公司之一，向全球客户销售清洁电力，并开发风能、太阳能、储能及电网基础设施。</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>从中国采购大型储能系统（直流侧）、磷酸铁锂电芯、储能变流器（PCS）及EMS能量管理系统。</t>
+          <t>大规模电网级储能系统（用于美国、澳大利亚、欧洲市场）、配套电池PCS/EMS、以及用于可再生能源混合项目的长时储能。</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>寻求具有海外项目经验（欧洲/北美）、通过CE/UL认证、能提供EPC配套服务的中国储能系统集成商或电芯厂商。</t>
+          <t>寻求具有全球供应链能力、能提供Tier-1电芯和系统集成、且具备国际项目融资支持能力的大型储能制造商。</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>法国、英国、美国、南非、智利</t>
+          <t>西班牙、英国、美国、巴西、墨西哥、澳大利亚</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>暂无在华分公司，但通过中国供应商（如比亚迪、宁德时代）进行采购</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola、NextEra Energy Resources、Engie</t>
+          <t>Enel Green Power, EDP Renováveis, NextEra Energy</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>全球可再生能源开发商前十，欧洲风电/光伏市场份额约5%</t>
+          <t>全球可再生能源装机容量约42GW，是全球前三大风电和光伏运营商。</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2025年与法国电网公司签署1.2GW储能项目框架协议，并启动在英国的3GWh电池储能项目。</t>
+          <t>2025年宣布在澳大利亚昆士兰州投建400MW/1600MWh的独立储能项目，预计2027年投运。</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Renewable Developer</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1528,83 +1528,83 @@
         </is>
       </c>
       <c r="R11" s="3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Large renewable developer with storage projects, open to global sourcing for cost efficiency.</t>
+          <t>Spanish utility giant with global storage projects, actively procuring batteries from multiple sources.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Acciona Energía</t>
+          <t>Enel Green Power</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.acciona-energia.com</t>
+          <t>https://www.enelgreenpower.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>马德里，西班牙</t>
+          <t>罗马，意大利</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>12000</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>约35亿欧元</t>
+          <t>约150亿欧元</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>西班牙跨国可再生能源巨头，销售风电、光伏电站电力，并提供储能系统解决方案及绿电采购协议（PPA）。</t>
+          <t>意大利国家电力公司（Enel）旗下可再生能源子公司，在全球开发并销售风电、太阳能、地热及储能项目电力。</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>从中国采购大型储能系统（50MW+）、电池电芯、PCS及用于其全球风光储一体化项目的配套设备。</t>
+          <t>电网级储能电池系统（主要针对美国、意大利、西班牙、澳大利亚市场）、集装箱式储能、以及用于混合电站的电池扩容。</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>寻找具备全球交付能力、有海外电站配套业绩、且能提供20年以上性能保证的中国储能系统集成商。</t>
+          <t>偏好能提供完整储能解决方案（电芯+PCS+EMS）、有美国UL认证和欧洲并网认证、且能支持长期质保的中国头部电池厂商。</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>西班牙、墨西哥、智利、澳大利亚、美国</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>在上海设有亚太采购代表处，负责设备询价和供应商审核。</t>
+          <t>意大利、西班牙、美国、巴西、智利、澳大利亚、南非</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Iberdrola, Enel Green Power, EDP Renewables</t>
+          <t>Iberdrola, EDP Renováveis, Acciona Energía</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>全球可再生能源开发商前十，西班牙市场份额第一。</t>
+          <t>全球可再生能源装机容量约60GW，是全球最大的私营可再生能源运营商之一。</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在智利建设1GWh储能项目，采用中国电芯，预计2026年投运。</t>
+          <t>2025年在美国德克萨斯州启动一个200MW/400MWh独立储能项目，并计划在2026年再投运1GW储能。</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1623,63 +1623,63 @@
         </is>
       </c>
       <c r="R12" s="3" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Spanish renewable developer with storage projects, known to source from Chinese manufacturers.</t>
+          <t>Italian renewable developer with large BESS installations, known to use Chinese battery suppliers.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eneco</t>
+          <t>Octopus Energy Generation</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://www.eneco.com</t>
+          <t>https://www.octopusenergy.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>鹿特丹，荷兰</t>
+          <t>London, UK</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>3500</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>约60亿欧元</t>
+          <t>3.2 billion GBP (2024)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>荷兰可持续能源公司，向欧洲客户销售绿色电力、天然气、热力及储能解决方案，并开发风能、太阳能和电池项目。</t>
+          <t>英国最大可再生能源投资与运营平台之一，管理超过5GW清洁能源资产，包括储能、风电、光伏，并运营电动汽车充电网络。</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>大型电池储能系统（用于平衡可再生能源）、工商业储能柜、以及虚拟电厂（VPP）中的分布式电池。</t>
+          <t>分布式储能系统（100kW-5MWh）、工商业储能柜、电池模组、充电桩配套储能（光储充一体化）。</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>寻找符合欧盟CE/电池护照标准、具备欧洲项目认证经验、能提供灵活OEM/ODM合作的储能系统集成商。</t>
+          <t>需要英国G99并网认证、MCS认证、灵活定制能力强的中国中小型储能系统集成商，支持OEM/ODM。</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>荷兰、比利时、德国、英国、法国</t>
+          <t>英国、德国、澳大利亚、日本</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1689,122 +1689,122 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Vattenfall, Ørsted, Essent (德国E.ON旗下)</t>
+          <t>E.ON UK, SSE Renewables, Centrica</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>荷兰可再生能源发电市场份额约15%，是荷兰最大的可持续能源零售商之一。</t>
+          <t>英国户用及工商业储能市场份额约8%（2025年）</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2025年与日本三井物产合作，在比利时启动一个50MW/100MWh的电池储能项目，以支持当地电网稳定。</t>
+          <t>2025年12月推出“储能+EV充电”套餐，采购500MWh电池；2026年1月与深圳某储能公司签订200MWh年度供货协议。</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>可再生能源开发商/EV充电运营商</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>英国</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>中型（高增长）</t>
         </is>
       </c>
       <c r="R13" s="3" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Dutch utility with growing BESS portfolio in Europe, seeking competitive suppliers.</t>
+          <t>英国储能+充电双重需求，采购灵活，对性价比高的中国产品接受度极高。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Shell Energy (Australia)</t>
+          <t>SSE Renewables</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.shellenergy.com.au</t>
+          <t>https://www.sserenewables.com</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>布里斯班，澳大利亚</t>
+          <t>珀斯，英国苏格兰</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>约1,200人</t>
+          <t>约1,500</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>约30亿澳元（2024年）</t>
+          <t>约15亿英镑</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>壳牌旗下澳大利亚能源零售与贸易公司，销售电力、天然气，并投资大型电池储能项目（如Riverside Energy Park）。</t>
+          <t>英国领先的可再生能源开发商，专注于海上风电、陆上风电和水电，并积极拓展电池储能项目，向英国电网销售清洁电力。</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>从中国采购大型储能电池系统（4小时以上长时储能）、电芯及储能电站运维备件。</t>
+          <t>采购英国电网级储能系统（50-200MW）、频率响应电池、以及用于风电配储的集成储能解决方案。</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>寻找具备澳洲CEC认证、有本地运维支持能力、能提供10年以上质保的中国储能系统供应商。</t>
+          <t>寻找有英国G99并网认证、能提供全生命周期维护、且在英国有本地服务团队的中国储能集成商。</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚、新西兰</t>
+          <t>英国、爱尔兰、挪威</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>暂无在华采购中心，但通过壳牌全球采购网络间接采购中国电池</t>
+          <t>暂无（通过英国本地工程公司间接采购中国设备）</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>AGL Energy、Origin Energy、EnergyAustralia</t>
+          <t>ScottishPower Renewables、Iberdrola、Equinor</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚工商业电力市场份额约10%，储能项目储备超2GWh</t>
+          <t>英国海上风电市场份额约15%，储能项目储备超2GW。</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2025年启动昆士兰州200MW/800MWh电池储能项目，预计2027年投运。</t>
+          <t>2025年获批在苏格兰建设600MW/2.4GWh电池储能项目，为英国最大独立储能项目之一。</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Energy Retailer</t>
+          <t>Renewable Developer</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -1813,93 +1813,93 @@
         </is>
       </c>
       <c r="R14" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Energy retailer with storage investments, known to source batteries from multiple vendors.</t>
+          <t>UK-based developer with large battery storage projects, open to international suppliers for competitive pricing.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Powercor</t>
+          <t>EDF Renewables</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.powercor.com.au</t>
+          <t>https://www.edf-renewables.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>墨尔本，澳大利亚</t>
+          <t>巴黎，法国</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>约5,000人</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>约20亿澳元</t>
+          <t>约50亿欧元（2024年）</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚维多利亚州最大的配电网络运营商，销售电网接入服务、分布式能源管理方案及社区电池储能项目。</t>
+          <t>法国电力集团旗下可再生能源子公司，开发、建设并运营风电、光伏及配套储能电站，销售电力及储能服务。</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>从中国采购配电网级储能系统（2-10MWh）、智能电表、变压器及电网侧电池储能设备。</t>
+          <t>从中国采购大型储能系统（直流侧）、磷酸铁锂电芯、储能变流器（PCS）及EMS能量管理系统。</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>需要符合澳大利亚CEC列名、具备高防护等级（IP65+）且能适应极端高温环境的中国储能设备供应商。</t>
+          <t>寻求具有海外项目经验（欧洲/北美）、通过CE/UL认证、能提供EPC配套服务的中国储能系统集成商或电芯厂商。</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>澳大利亚（维多利亚州）</t>
+          <t>法国、英国、美国、南非、智利</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>暂无，通过本地分销商采购。</t>
+          <t>暂无在华分公司，但通过中国供应商（如比亚迪、宁德时代）进行采购</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>AusNet Services, CitiPower, United Energy</t>
+          <t>Iberdrola、NextEra Energy Resources、Engie</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>维州配电市场份额约50%，澳洲电网侧储能试点项目主要参与者。</t>
+          <t>全球可再生能源开发商前十，欧洲风电/光伏市场份额约5%</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2025年启动“社区电池计划”，采购50MWh分布式储能设备用于缓解电网拥堵。</t>
+          <t>2025年与法国电网公司签署1.2GW储能项目框架协议，并启动在英国的3GWh电池储能项目。</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Utility</t>
+          <t>Renewable Developer</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>US</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
@@ -1908,93 +1908,93 @@
         </is>
       </c>
       <c r="R15" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Australian distribution utility with storage projects, open to global suppliers.</t>
+          <t>Large renewable developer with storage projects, open to global sourcing for cost efficiency.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tesla Energy</t>
+          <t>Acciona Energía</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.tesla.com/energy</t>
+          <t>https://www.acciona-energia.com</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>奥斯汀，美国</t>
+          <t>马德里，西班牙</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>约2,000人（能源部门）</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元（2024年能源业务）</t>
+          <t>约35亿欧元</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>销售Megapack（大型储能系统）、Powerwall（户用电池）及太阳能屋顶，提供电网级储能解决方案。</t>
+          <t>西班牙跨国可再生能源巨头，销售风电、光伏电站电力，并提供储能系统解决方案及绿电采购协议（PPA）。</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>从中国采购LFP电池电芯（主要来自宁德时代）、储能系统结构件、电力电子组件（逆变器/变流器）。</t>
+          <t>从中国采购大型储能系统（50MW+）、电池电芯、PCS及用于其全球风光储一体化项目的配套设备。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>寻找具备高性价比、大规模稳定供货能力、通过UL9540A认证的中国电芯制造商，以及精密钣金和热管理部件供应商。</t>
+          <t>寻找具备全球交付能力、有海外电站配套业绩、且能提供20年以上性能保证的中国储能系统集成商。</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>美国、澳大利亚、英国、德国、日本</t>
+          <t>西班牙、墨西哥、智利、澳大利亚、美国</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>上海超级工厂（Model 3/Y），能源业务在华暂无独立采购中心，但电芯采购自宁德时代（福建）</t>
+          <t>在上海设有亚太采购代表处，负责设备询价和供应商审核。</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Fluence、比亚迪储能、阳光电源</t>
+          <t>Iberdrola, Enel Green Power, EDP Renewables</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>全球电网级储能市场份额约15-20%，Megapack为北美最畅销大型储能产品</t>
+          <t>全球可再生能源开发商前十，西班牙市场份额第一。</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2025年推出Megapack 3，单机容量提升至4MWh，并宣布在加州扩建储能超级工厂。</t>
+          <t>2025年宣布在智利建设1GWh储能项目，采用中国电芯，预计2026年投运。</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Microgrid Developer</t>
+          <t>Renewable Developer</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -2003,93 +2003,93 @@
         </is>
       </c>
       <c r="R16" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Major BESS player but primarily uses own batteries, less likely to buy Chinese products.</t>
+          <t>Spanish renewable developer with storage projects, known to source from Chinese manufacturers.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Lightsource bp</t>
+          <t>Eneco</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.lightsourcebp.com</t>
+          <t>https://www.eneco.com</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>伦敦，英国</t>
+          <t>鹿特丹，荷兰</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>约1,000人</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元（2024年）</t>
+          <t>约60亿欧元</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>bp旗下太阳能及储能开发商，销售清洁电力，开发光伏+储能项目，并提供能源管理服务。</t>
+          <t>荷兰可持续能源公司，向欧洲客户销售绿色电力、天然气、热力及储能解决方案，并开发风能、太阳能和电池项目。</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>从中国采购光伏+储能一体化系统（DC-coupled）、LFP电池、逆变器及跟踪支架。</t>
+          <t>大型电池储能系统（用于平衡可再生能源）、工商业储能柜、以及虚拟电厂（VPP）中的分布式电池。</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>寻求有全球项目交付能力、具备IEC/UL认证、能提供融资支持的中国新能源设备供应商。</t>
+          <t>寻找符合欧盟CE/电池护照标准、具备欧洲项目认证经验、能提供灵活OEM/ODM合作的储能系统集成商。</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>美国、英国、西班牙、希腊、印度</t>
+          <t>荷兰、比利时、德国、英国、法国</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>暂无在华分公司，但通过bp中国办公室进行部分采购协调</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>NextEra Energy、Brookfield Renewable、TotalEnergies Renewables</t>
+          <t>Vattenfall, Ørsted, Essent (德国E.ON旗下)</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>全球太阳能开发商前十，累计开发超10GW光伏项目</t>
+          <t>荷兰可再生能源发电市场份额约15%，是荷兰最大的可持续能源零售商之一。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2025年与bp合作在美国德州开发1.5GW光伏+1GWh储能项目，并宣布进入波兰市场。</t>
+          <t>2025年与日本三井物产合作，在比利时启动一个50MW/100MWh的电池储能项目，以支持当地电网稳定。</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Solar Installer</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -2098,93 +2098,93 @@
         </is>
       </c>
       <c r="R17" s="3" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Global solar developer with storage projects, potential buyer of Chinese BESS.</t>
+          <t>Dutch utility with growing BESS portfolio in Europe, seeking competitive suppliers.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BayWa r.e.</t>
+          <t>Shell Energy (Australia)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.baywa-re.com</t>
+          <t>https://www.shellenergy.com.au</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>慕尼黑，德国</t>
+          <t>布里斯班，澳大利亚</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>约1,200人</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>约50亿欧元</t>
+          <t>约30亿澳元（2024年）</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>全球领先的可再生能源开发商、服务和分销商，销售太阳能组件、逆变器、储能系统及提供项目开发、运维服务。</t>
+          <t>壳牌旗下澳大利亚能源零售与贸易公司，销售电力、天然气，并投资大型电池储能项目（如Riverside Energy Park）。</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>从中国采购磷酸铁锂储能电芯、家用及工商业储能整机、光伏组件及逆变器，用于其全球项目交付和分销业务。</t>
+          <t>从中国采购大型储能电池系统（4小时以上长时储能）、电芯及储能电站运维备件。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>寻找具备TÜV/UL认证、产能稳定、成本竞争力强且能提供长期质保的中国电池和储能系统制造商。</t>
+          <t>寻找具备澳洲CEC认证、有本地运维支持能力、能提供10年以上质保的中国储能系统供应商。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>德国、美国、澳大利亚、西班牙、英国</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>在上海设有亚太区办公室，负责采购和供应商管理。</t>
+          <t>澳大利亚、新西兰</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>暂无在华采购中心，但通过壳牌全球采购网络间接采购中国电池</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>JUWI, Enerparc, ib vogt</t>
+          <t>AGL Energy、Origin Energy、EnergyAustralia</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>欧洲光伏及储能分销市场前五，全球可再生能源EPC服务商前十。</t>
+          <t>澳大利亚工商业电力市场份额约10%，储能项目储备超2GWh</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布与宁德时代签署长期供货协议，用于其欧洲大型储能项目。</t>
+          <t>2025年启动昆士兰州200MW/800MWh电池储能项目，预计2027年投运。</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Solar Installer</t>
+          <t>Energy Retailer</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2193,301 +2193,776 @@
         </is>
       </c>
       <c r="R18" s="3" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Renewable energy company with storage solutions, actively seeking competitive battery suppliers.</t>
+          <t>Energy retailer with storage investments, known to source batteries from multiple vendors.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sonnen GmbH</t>
+          <t>Powercor</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.sonnen.de</t>
+          <t>https://www.powercor.com.au</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>慕尼黑，德国</t>
+          <t>墨尔本，澳大利亚</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>约3亿欧元</t>
+          <t>约20亿澳元</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>智能家庭储能系统制造商，销售sonnenBatterie系列家用电池、虚拟电厂平台及能源社区服务。</t>
+          <t>澳大利亚维多利亚州最大的配电网络运营商，销售电网接入服务、分布式能源管理方案及社区电池储能项目。</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>从中国采购高循环寿命的磷酸铁锂电芯、BMS（电池管理系统）以及家用储能一体机代工（OEM/ODM）。</t>
+          <t>从中国采购配电网级储能系统（2-10MWh）、智能电表、变压器及电网侧电池储能设备。</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>偏好有车规级制造经验、电芯一致性高、能配合欧洲本地售后服务的中国电池企业。</t>
+          <t>需要符合澳大利亚CEC列名、具备高防护等级（IP65+）且能适应极端高温环境的中国储能设备供应商。</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>德国、美国、英国、意大利、澳大利亚</t>
+          <t>澳大利亚（维多利亚州）</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>暂无，但通过深圳/东莞的代工厂进行间接采购。</t>
+          <t>暂无，通过本地分销商采购。</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Tesla (Powerwall), BYD (B-Box), E3/DC</t>
+          <t>AusNet Services, CitiPower, United Energy</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>德国户用储能市场份额约20%，全球高端家用储能品牌前三。</t>
+          <t>维州配电市场份额约50%，澳洲电网侧储能试点项目主要参与者。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2025年推出sonnenPro 2.0，采用中国电芯，主打社区级虚拟电厂功能。</t>
+          <t>2025年启动“社区电池计划”，采购50MWh分布式储能设备用于缓解电网拥堵。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Microgrid Developer</t>
+          <t>Utility</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Medium (100-1000)</t>
-        </is>
-      </c>
-      <c r="R19" s="5" t="n">
-        <v>65</v>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>75</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Residential storage provider, but uses own batteries, may buy cells from Chinese suppliers.</t>
+          <t>Australian distribution utility with storage projects, open to global suppliers.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Green Investment Group</t>
+          <t>Eneco (Shell-backed)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.greeninvestmentgroup.com</t>
+          <t>https://www.eneco.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>伦敦，英国</t>
+          <t>Rotterdam, Netherlands</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>约5亿英镑（投资组合收入）</t>
+          <t>6.5 billion EUR (2024)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>麦格理集团旗下的绿色基础设施投资机构，投资并开发大型风电、太阳能和储能项目，销售项目股权和电力资产。</t>
+          <t>荷兰领先的可持续能源公司，壳牌全资子公司，运营风电、光伏、储能及电动汽车充电网络，业务覆盖荷兰、比利时、德国。</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>为其投资的储能项目集中采购大型集装箱式储能系统（直流侧电池舱+交流侧PCS），以及长期运维服务。</t>
+          <t>储能电池系统（电网级和工商业）、电池租赁服务、光储充一体化设备、虚拟电厂（VPP）配套储能。</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>寻找具备海外大型项目交付经验（如美国、英国市场）、具备UL9540A认证且能提供项目融资支持的中国储能集成商。</t>
+          <t>需要CE认证、荷兰电网认证（Netcode），有欧洲成功案例的中国供应商，尤其欢迎有液冷储能技术的企业。</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>英国、澳大利亚、美国、韩国、中国台湾</t>
+          <t>荷兰、比利时、德国、法国</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>暂无，但通过麦格理集团香港办公室协调亚洲采购。</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>NextEra Energy Resources, Copenhagen Infrastructure Partners, Foresight Group</t>
+          <t>Vattenfall, ENGIE, TotalEnergies</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>全球绿色基础设施投资领域前五，管理资产超100亿英镑。</t>
+          <t>荷兰储能市场份额约20%，欧洲工商业储能前五</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布收购英国1.2GW储能项目组合，计划2026年启动设备招标。</t>
+          <t>2025年11月启用荷兰最大储能站（300MW/600MWh）；2026年2月发布2026-2028年储能采购框架，预计采购1.5GWh，明确考虑中国供应商。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Renewable Developer</t>
+          <t>电力公司/EV充电运营商</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>荷兰</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Medium (100-1000)</t>
-        </is>
-      </c>
-      <c r="R20" s="5" t="n">
-        <v>60</v>
+          <t>大型（壳牌子公司）</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>75</v>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure investor with storage projects, potential buyer of Chinese BESS.</t>
+          <t>荷兰储能市场核心买家，壳牌背景资金雄厚，2026年有明确采购计划，中国产品竞争力强。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Tesla Energy</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tesla.com/energy</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>奥斯汀，美国</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>约2,000人（能源部门）</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>约60亿美元（2024年能源业务）</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>销售Megapack（大型储能系统）、Powerwall（户用电池）及太阳能屋顶，提供电网级储能解决方案。</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>从中国采购LFP电池电芯（主要来自宁德时代）、储能系统结构件、电力电子组件（逆变器/变流器）。</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>寻找具备高性价比、大规模稳定供货能力、通过UL9540A认证的中国电芯制造商，以及精密钣金和热管理部件供应商。</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>美国、澳大利亚、英国、德国、日本</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>上海超级工厂（Model 3/Y），能源业务在华暂无独立采购中心，但电芯采购自宁德时代（福建）</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Fluence、比亚迪储能、阳光电源</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>全球电网级储能市场份额约15-20%，Megapack为北美最畅销大型储能产品</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2025年推出Megapack 3，单机容量提升至4MWh，并宣布在加州扩建储能超级工厂。</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Microgrid Developer</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Major BESS player but primarily uses own batteries, less likely to buy Chinese products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Lightsource bp</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lightsourcebp.com</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>伦敦，英国</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>约1,000人</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>约15亿美元（2024年）</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>bp旗下太阳能及储能开发商，销售清洁电力，开发光伏+储能项目，并提供能源管理服务。</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>从中国采购光伏+储能一体化系统（DC-coupled）、LFP电池、逆变器及跟踪支架。</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>寻求有全球项目交付能力、具备IEC/UL认证、能提供融资支持的中国新能源设备供应商。</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>美国、英国、西班牙、希腊、印度</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>暂无在华分公司，但通过bp中国办公室进行部分采购协调</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>NextEra Energy、Brookfield Renewable、TotalEnergies Renewables</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>全球太阳能开发商前十，累计开发超10GW光伏项目</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2025年与bp合作在美国德州开发1.5GW光伏+1GWh储能项目，并宣布进入波兰市场。</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Solar Installer</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Global solar developer with storage projects, potential buyer of Chinese BESS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>BayWa r.e.</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.baywa-re.com</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>慕尼黑，德国</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>4500</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>约50亿欧元</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>全球领先的可再生能源开发商、服务和分销商，销售太阳能组件、逆变器、储能系统及提供项目开发、运维服务。</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>从中国采购磷酸铁锂储能电芯、家用及工商业储能整机、光伏组件及逆变器，用于其全球项目交付和分销业务。</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>寻找具备TÜV/UL认证、产能稳定、成本竞争力强且能提供长期质保的中国电池和储能系统制造商。</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>德国、美国、澳大利亚、西班牙、英国</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>在上海设有亚太区办公室，负责采购和供应商管理。</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>JUWI, Enerparc, ib vogt</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>欧洲光伏及储能分销市场前五，全球可再生能源EPC服务商前十。</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布与宁德时代签署长期供货协议，用于其欧洲大型储能项目。</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Solar Installer</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>Renewable energy company with storage solutions, actively seeking competitive battery suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Sonnen GmbH</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sonnen.de</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>慕尼黑，德国</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>约3亿欧元</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>智能家庭储能系统制造商，销售sonnenBatterie系列家用电池、虚拟电厂平台及能源社区服务。</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>从中国采购高循环寿命的磷酸铁锂电芯、BMS（电池管理系统）以及家用储能一体机代工（OEM/ODM）。</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>偏好有车规级制造经验、电芯一致性高、能配合欧洲本地售后服务的中国电池企业。</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>德国、美国、英国、意大利、澳大利亚</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>暂无，但通过深圳/东莞的代工厂进行间接采购。</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Tesla (Powerwall), BYD (B-Box), E3/DC</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>德国户用储能市场份额约20%，全球高端家用储能品牌前三。</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2025年推出sonnenPro 2.0，采用中国电芯，主打社区级虚拟电厂功能。</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Microgrid Developer</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Medium (100-1000)</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>Residential storage provider, but uses own batteries, may buy cells from Chinese suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Green Investment Group</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.greeninvestmentgroup.com</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>伦敦，英国</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>约5亿英镑（投资组合收入）</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>麦格理集团旗下的绿色基础设施投资机构，投资并开发大型风电、太阳能和储能项目，销售项目股权和电力资产。</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>为其投资的储能项目集中采购大型集装箱式储能系统（直流侧电池舱+交流侧PCS），以及长期运维服务。</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>寻找具备海外大型项目交付经验（如美国、英国市场）、具备UL9540A认证且能提供项目融资支持的中国储能集成商。</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>英国、澳大利亚、美国、韩国、中国台湾</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>暂无，但通过麦格理集团香港办公室协调亚洲采购。</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>NextEra Energy Resources, Copenhagen Infrastructure Partners, Foresight Group</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>全球绿色基础设施投资领域前五，管理资产超100亿英镑。</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布收购英国1.2GW储能项目组合，计划2026年启动设备招标。</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Renewable Developer</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>Medium (100-1000)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>Infrastructure investor with storage projects, potential buyer of Chinese BESS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Sungrow Power Supply Co., Ltd.</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>https://www.sungrowpower.com</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>1997</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>合肥，中国</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>约10,000人</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>约70亿美元（2024年）</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>全球领先的逆变器和储能系统供应商，销售光伏逆变器、储能变流器（PCS）及交直流储能系统，产品覆盖户用至GW级电站。</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>从中国采购高能量密度锂电池（LFP）、BMS（电池管理系统）、热管理组件及储能集装箱集成部件。</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>寻求具备大规模量产能力、电芯一致性高、通过UL/IEC认证的中国电池及核心部件供应商，支持OEM/ODM定制。</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>中国、美国、德国、澳大利亚、巴西</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>总部及主要生产基地在中国合肥，另在深圳、上海设有研发中心</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>华为数字能源、比亚迪储能、宁德时代（CATL）</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>全球光伏逆变器出货量第一（约30%），储能系统出货量全球前三</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>2025年推出新一代液冷储能系统PowerTitan 2.0，并宣布在沙特建设5GW储能制造基地。</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Solar Installer</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr">
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R21" s="5" t="n">
+      <c r="R26" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="S26" s="2" t="inlineStr">
         <is>
           <t>Chinese manufacturer but also a buyer of batteries for system integration, though not a target buyer.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S21"/>
+  <autoFilter ref="A1:S26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>